<commit_message>
Fix lvl 45 SK
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/27_SiegeKitItem/SiegeKitItem.xlsx
+++ b/gu_in/Item.edf/27_SiegeKitItem/SiegeKitItem.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3694E5B1-754B-4F4B-B65C-B6B81FFF2ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61877373-6E53-407C-946A-D19F0CEB61B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SiegeKitItem" sheetId="1" r:id="rId1"/>
@@ -586,7 +586,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -595,8 +595,21 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -611,6 +624,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="42"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -644,17 +662,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -671,9 +694,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -711,9 +734,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -746,9 +769,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -781,9 +821,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -958,62 +1015,62 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AY33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="7" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="8" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="9" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="12" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="9" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="12" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="9" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="9" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="9" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="4.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1168,7 +1225,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1321,7 +1378,7 @@
       </c>
       <c r="AY2" s="2"/>
     </row>
-    <row r="3" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>55</v>
       </c>
@@ -1474,7 +1531,7 @@
       </c>
       <c r="AY3" s="2"/>
     </row>
-    <row r="4" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>58</v>
       </c>
@@ -1627,160 +1684,160 @@
       </c>
       <c r="AY4" s="2"/>
     </row>
-    <row r="5" spans="1:51" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:51" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="3">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D5" s="3">
-        <v>4</v>
-      </c>
-      <c r="E5" s="3" t="s">
+      <c r="B5" s="5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="6">
         <v>285</v>
       </c>
-      <c r="G5" s="3">
-        <v>0</v>
-      </c>
-      <c r="H5" s="3">
+      <c r="G5" s="5">
+        <v>0</v>
+      </c>
+      <c r="H5" s="5">
         <v>7</v>
       </c>
-      <c r="I5" s="3">
-        <v>0</v>
-      </c>
-      <c r="J5" s="3" t="s">
+      <c r="I5" s="5">
+        <v>0</v>
+      </c>
+      <c r="J5" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="5">
+        <v>45</v>
+      </c>
+      <c r="L5" s="5">
+        <v>-1</v>
+      </c>
+      <c r="M5" s="5">
+        <v>-1</v>
+      </c>
+      <c r="N5" s="5">
+        <v>0</v>
+      </c>
+      <c r="O5" s="5">
+        <v>-1</v>
+      </c>
+      <c r="P5" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>0</v>
+      </c>
+      <c r="R5" s="5">
+        <v>2100</v>
+      </c>
+      <c r="S5" s="5">
+        <v>0</v>
+      </c>
+      <c r="T5" s="5">
+        <v>0</v>
+      </c>
+      <c r="U5" s="5">
+        <v>0</v>
+      </c>
+      <c r="V5" s="5">
+        <v>0</v>
+      </c>
+      <c r="W5" s="5">
+        <v>105</v>
+      </c>
+      <c r="X5" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="5">
+        <v>1000</v>
+      </c>
+      <c r="Z5" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="6">
+        <v>1</v>
+      </c>
+      <c r="AC5" s="5">
+        <v>1</v>
+      </c>
+      <c r="AD5" s="5">
         <v>50</v>
       </c>
-      <c r="L5" s="3">
-        <v>-1</v>
-      </c>
-      <c r="M5" s="3">
-        <v>-1</v>
-      </c>
-      <c r="N5" s="3">
-        <v>0</v>
-      </c>
-      <c r="O5" s="3">
-        <v>-1</v>
-      </c>
-      <c r="P5" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="3">
-        <v>0</v>
-      </c>
-      <c r="R5" s="3">
-        <v>2100</v>
-      </c>
-      <c r="S5" s="3">
-        <v>0</v>
-      </c>
-      <c r="T5" s="3">
-        <v>0</v>
-      </c>
-      <c r="U5" s="3">
-        <v>0</v>
-      </c>
-      <c r="V5" s="3">
-        <v>0</v>
-      </c>
-      <c r="W5" s="3">
-        <v>105</v>
-      </c>
-      <c r="X5" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y5" s="3">
-        <v>1000</v>
-      </c>
-      <c r="Z5" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="2">
-        <v>1</v>
-      </c>
-      <c r="AC5" s="3">
-        <v>1</v>
-      </c>
-      <c r="AD5" s="3">
-        <v>50</v>
-      </c>
-      <c r="AE5" s="3">
+      <c r="AE5" s="5">
         <v>-550</v>
       </c>
-      <c r="AF5" s="3">
-        <v>1</v>
-      </c>
-      <c r="AG5" s="3">
+      <c r="AF5" s="5">
+        <v>1</v>
+      </c>
+      <c r="AG5" s="5">
         <v>6</v>
       </c>
-      <c r="AH5" s="3">
-        <v>0.40000000596046448</v>
-      </c>
-      <c r="AI5" s="3">
+      <c r="AH5" s="5">
+        <v>0.300000005960464</v>
+      </c>
+      <c r="AI5" s="5">
         <v>5</v>
       </c>
-      <c r="AJ5" s="3">
+      <c r="AJ5" s="5">
         <v>0.10000000149011612</v>
       </c>
-      <c r="AK5" s="3">
+      <c r="AK5" s="5">
         <v>21</v>
       </c>
-      <c r="AL5" s="3">
+      <c r="AL5" s="5">
         <v>0.10000000149011612</v>
       </c>
-      <c r="AM5" s="3">
+      <c r="AM5" s="5">
         <v>3</v>
       </c>
-      <c r="AN5" s="3">
-        <v>20</v>
-      </c>
-      <c r="AO5" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP5" s="3">
-        <v>1</v>
-      </c>
-      <c r="AQ5" s="3">
-        <v>1</v>
-      </c>
-      <c r="AR5" s="3">
-        <v>1</v>
-      </c>
-      <c r="AS5" s="3">
-        <v>1</v>
-      </c>
-      <c r="AT5" s="2">
-        <v>1</v>
-      </c>
-      <c r="AU5" s="3">
-        <v>0</v>
-      </c>
-      <c r="AV5" s="2" t="s">
+      <c r="AN5" s="5">
+        <v>10</v>
+      </c>
+      <c r="AO5" s="6">
+        <v>0</v>
+      </c>
+      <c r="AP5" s="5">
+        <v>1</v>
+      </c>
+      <c r="AQ5" s="5">
+        <v>1</v>
+      </c>
+      <c r="AR5" s="5">
+        <v>1</v>
+      </c>
+      <c r="AS5" s="5">
+        <v>1</v>
+      </c>
+      <c r="AT5" s="6">
+        <v>1</v>
+      </c>
+      <c r="AU5" s="5">
+        <v>0</v>
+      </c>
+      <c r="AV5" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="AW5" s="3">
+      <c r="AW5" s="5">
         <v>11</v>
       </c>
-      <c r="AX5" s="3">
-        <v>0</v>
-      </c>
-      <c r="AY5" s="2"/>
+      <c r="AX5" s="5">
+        <v>0</v>
+      </c>
+      <c r="AY5" s="6"/>
     </row>
-    <row r="6" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>63</v>
       </c>
@@ -1933,7 +1990,7 @@
       </c>
       <c r="AY6" s="2"/>
     </row>
-    <row r="7" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>65</v>
       </c>
@@ -2086,7 +2143,7 @@
       </c>
       <c r="AY7" s="2"/>
     </row>
-    <row r="8" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>68</v>
       </c>
@@ -2239,7 +2296,7 @@
       </c>
       <c r="AY8" s="2"/>
     </row>
-    <row r="9" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>70</v>
       </c>
@@ -2392,7 +2449,7 @@
       </c>
       <c r="AY9" s="2"/>
     </row>
-    <row r="10" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>73</v>
       </c>
@@ -2545,7 +2602,7 @@
       </c>
       <c r="AY10" s="2"/>
     </row>
-    <row r="11" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>75</v>
       </c>
@@ -2698,7 +2755,7 @@
       </c>
       <c r="AY11" s="2"/>
     </row>
-    <row r="12" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>77</v>
       </c>
@@ -2851,7 +2908,7 @@
       </c>
       <c r="AY12" s="2"/>
     </row>
-    <row r="13" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>80</v>
       </c>
@@ -3004,7 +3061,7 @@
       </c>
       <c r="AY13" s="2"/>
     </row>
-    <row r="14" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>82</v>
       </c>
@@ -3157,7 +3214,7 @@
       </c>
       <c r="AY14" s="2"/>
     </row>
-    <row r="15" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -3310,7 +3367,7 @@
       </c>
       <c r="AY15" s="2"/>
     </row>
-    <row r="16" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>86</v>
       </c>
@@ -3463,7 +3520,7 @@
       </c>
       <c r="AY16" s="2"/>
     </row>
-    <row r="17" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>88</v>
       </c>
@@ -3616,7 +3673,7 @@
       </c>
       <c r="AY17" s="2"/>
     </row>
-    <row r="18" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>90</v>
       </c>
@@ -3769,7 +3826,7 @@
       </c>
       <c r="AY18" s="2"/>
     </row>
-    <row r="19" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>93</v>
       </c>
@@ -3922,7 +3979,7 @@
       </c>
       <c r="AY19" s="2"/>
     </row>
-    <row r="20" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>95</v>
       </c>
@@ -4075,7 +4132,7 @@
       </c>
       <c r="AY20" s="2"/>
     </row>
-    <row r="21" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>97</v>
       </c>
@@ -4228,7 +4285,7 @@
       </c>
       <c r="AY21" s="2"/>
     </row>
-    <row r="22" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>99</v>
       </c>
@@ -4381,7 +4438,7 @@
       </c>
       <c r="AY22" s="2"/>
     </row>
-    <row r="23" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>101</v>
       </c>
@@ -4534,7 +4591,7 @@
       </c>
       <c r="AY23" s="2"/>
     </row>
-    <row r="24" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>103</v>
       </c>
@@ -4687,7 +4744,7 @@
       </c>
       <c r="AY24" s="2"/>
     </row>
-    <row r="25" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>105</v>
       </c>
@@ -4840,7 +4897,7 @@
       </c>
       <c r="AY25" s="2"/>
     </row>
-    <row r="26" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>107</v>
       </c>
@@ -4993,7 +5050,7 @@
       </c>
       <c r="AY26" s="2"/>
     </row>
-    <row r="27" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>109</v>
       </c>
@@ -5146,7 +5203,7 @@
       </c>
       <c r="AY27" s="2"/>
     </row>
-    <row r="28" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>111</v>
       </c>
@@ -5299,7 +5356,7 @@
       </c>
       <c r="AY28" s="2"/>
     </row>
-    <row r="29" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>113</v>
       </c>
@@ -5452,7 +5509,7 @@
       </c>
       <c r="AY29" s="2"/>
     </row>
-    <row r="30" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>115</v>
       </c>
@@ -5605,7 +5662,7 @@
       </c>
       <c r="AY30" s="2"/>
     </row>
-    <row r="31" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>117</v>
       </c>
@@ -5758,7 +5815,7 @@
       </c>
       <c r="AY31" s="2"/>
     </row>
-    <row r="32" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>119</v>
       </c>
@@ -5911,7 +5968,7 @@
       </c>
       <c r="AY32" s="2"/>
     </row>
-    <row r="33" spans="1:51" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>122</v>
       </c>
@@ -6073,59 +6130,59 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:BH33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="9" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="6" bestFit="1" customWidth="1"/>
     <col min="30" max="31" width="7" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="39" max="42" width="9" bestFit="1" customWidth="1"/>
-    <col min="43" max="45" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="43" max="45" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="46" max="47" width="12" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="4.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>125</v>
       </c>
@@ -6307,7 +6364,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>SiegeKitItem!A2</f>
         <v>Code</v>
@@ -6528,7 +6585,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f>SiegeKitItem!A3</f>
         <v>sklu001</v>
@@ -6750,7 +6807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f>SiegeKitItem!A4</f>
         <v>sklu002</v>
@@ -6972,7 +7029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f>SiegeKitItem!A5</f>
         <v>sklu003</v>
@@ -6983,11 +7040,11 @@
       </c>
       <c r="C5" s="1" t="str">
         <f>SiegeKitItem!C5</f>
-        <v>411D03</v>
+        <v>411D01</v>
       </c>
       <c r="D5">
         <f>SiegeKitItem!D5</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E5" s="1" t="str">
         <f>SiegeKitItem!J5</f>
@@ -7081,7 +7138,7 @@
       </c>
       <c r="AC5">
         <f>SiegeKitItem!K5</f>
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="AD5">
         <f>SiegeKitItem!M5</f>
@@ -7142,7 +7199,7 @@
       </c>
       <c r="AT5">
         <f>SiegeKitItem!AH5</f>
-        <v>0.40000000596046448</v>
+        <v>0.300000005960464</v>
       </c>
       <c r="AU5">
         <f>SiegeKitItem!AJ5</f>
@@ -7154,7 +7211,7 @@
       </c>
       <c r="AW5">
         <f>SiegeKitItem!AN5</f>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="AX5">
         <f>SiegeKitItem!AW5</f>
@@ -7194,7 +7251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f>SiegeKitItem!A6</f>
         <v>sklu004</v>
@@ -7416,7 +7473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f>SiegeKitItem!A7</f>
         <v>sklu005</v>
@@ -7638,7 +7695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f>SiegeKitItem!A8</f>
         <v>sklu006</v>
@@ -7860,7 +7917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f>SiegeKitItem!A9</f>
         <v>sklu007</v>
@@ -8082,7 +8139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f>SiegeKitItem!A10</f>
         <v>sklu008</v>
@@ -8304,7 +8361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f>SiegeKitItem!A11</f>
         <v>sklu009</v>
@@ -8526,7 +8583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f>SiegeKitItem!A12</f>
         <v>sklu010</v>
@@ -8748,7 +8805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f>SiegeKitItem!A13</f>
         <v>sklu011</v>
@@ -8970,7 +9027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f>SiegeKitItem!A14</f>
         <v>sklu012</v>
@@ -9192,7 +9249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f>SiegeKitItem!A15</f>
         <v>sklu013</v>
@@ -9414,7 +9471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f>SiegeKitItem!A16</f>
         <v>sklu014</v>
@@ -9636,7 +9693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f>SiegeKitItem!A17</f>
         <v>sklu015</v>
@@ -9858,7 +9915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f>SiegeKitItem!A18</f>
         <v>sklu016</v>
@@ -10080,7 +10137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f>SiegeKitItem!A19</f>
         <v>sklu017</v>
@@ -10302,7 +10359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f>SiegeKitItem!A20</f>
         <v>sklu018</v>
@@ -10524,7 +10581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f>SiegeKitItem!A21</f>
         <v>sklu019</v>
@@ -10746,7 +10803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f>SiegeKitItem!A22</f>
         <v>sklu020</v>
@@ -10968,7 +11025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f>SiegeKitItem!A23</f>
         <v>sklu021</v>
@@ -11190,7 +11247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f>SiegeKitItem!A24</f>
         <v>sklu022</v>
@@ -11412,7 +11469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f>SiegeKitItem!A25</f>
         <v>sklu023</v>
@@ -11634,7 +11691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f>SiegeKitItem!A26</f>
         <v>sklu024</v>
@@ -11856,7 +11913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f>SiegeKitItem!A27</f>
         <v>sklu025</v>
@@ -12078,7 +12135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f>SiegeKitItem!A28</f>
         <v>sklu026</v>
@@ -12300,7 +12357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f>SiegeKitItem!A29</f>
         <v>sklu027</v>
@@ -12522,7 +12579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f>SiegeKitItem!A30</f>
         <v>sklu028</v>
@@ -12744,7 +12801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f>SiegeKitItem!A31</f>
         <v>sklu029</v>
@@ -12966,7 +13023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f>SiegeKitItem!A32</f>
         <v>sklu030</v>
@@ -13188,7 +13245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f>SiegeKitItem!A33</f>
         <v>skbal01</v>
@@ -13419,9 +13476,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -13432,7 +13489,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>130</v>
       </c>
@@ -13441,7 +13498,7 @@
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>0</v>
       </c>
@@ -13450,7 +13507,7 @@
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>1</v>
       </c>
@@ -13459,7 +13516,7 @@
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>2</v>
       </c>
@@ -13468,7 +13525,7 @@
       </c>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>3</v>
       </c>
@@ -13477,7 +13534,7 @@
       </c>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>4</v>
       </c>
@@ -13486,7 +13543,7 @@
       </c>
       <c r="C7" s="2"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>5</v>
       </c>
@@ -13495,7 +13552,7 @@
       </c>
       <c r="C8" s="2"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>6</v>
       </c>
@@ -13504,7 +13561,7 @@
       </c>
       <c r="C9" s="2"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>7</v>
       </c>
@@ -13513,7 +13570,7 @@
       </c>
       <c r="C10" s="2"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>8</v>
       </c>
@@ -13522,7 +13579,7 @@
       </c>
       <c r="C11" s="2"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>9</v>
       </c>
@@ -13531,7 +13588,7 @@
       </c>
       <c r="C12" s="2"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>10</v>
       </c>
@@ -13540,7 +13597,7 @@
       </c>
       <c r="C13" s="2"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>11</v>
       </c>
@@ -13549,7 +13606,7 @@
       </c>
       <c r="C14" s="2"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>12</v>
       </c>
@@ -13558,7 +13615,7 @@
       </c>
       <c r="C15" s="2"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>13</v>
       </c>
@@ -13567,7 +13624,7 @@
       </c>
       <c r="C16" s="2"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>14</v>
       </c>
@@ -13576,7 +13633,7 @@
       </c>
       <c r="C17" s="2"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>15</v>
       </c>
@@ -13585,7 +13642,7 @@
       </c>
       <c r="C18" s="2"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>16</v>
       </c>
@@ -13594,7 +13651,7 @@
       </c>
       <c r="C19" s="2"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>17</v>
       </c>
@@ -13603,7 +13660,7 @@
       </c>
       <c r="C20" s="2"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>18</v>
       </c>
@@ -13612,7 +13669,7 @@
       </c>
       <c r="C21" s="2"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>19</v>
       </c>
@@ -13621,7 +13678,7 @@
       </c>
       <c r="C22" s="2"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>20</v>
       </c>
@@ -13630,7 +13687,7 @@
       </c>
       <c r="C23" s="2"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>21</v>
       </c>
@@ -13639,7 +13696,7 @@
       </c>
       <c r="C24" s="2"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>22</v>
       </c>
@@ -13648,7 +13705,7 @@
       </c>
       <c r="C25" s="2"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>23</v>
       </c>
@@ -13657,7 +13714,7 @@
       </c>
       <c r="C26" s="2"/>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>24</v>
       </c>
@@ -13666,7 +13723,7 @@
       </c>
       <c r="C27" s="2"/>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>25</v>
       </c>
@@ -13675,7 +13732,7 @@
       </c>
       <c r="C28" s="2"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>26</v>
       </c>
@@ -13684,7 +13741,7 @@
       </c>
       <c r="C29" s="2"/>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>27</v>
       </c>
@@ -13693,7 +13750,7 @@
       </c>
       <c r="C30" s="2"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>28</v>
       </c>
@@ -13702,7 +13759,7 @@
       </c>
       <c r="C31" s="2"/>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>29</v>
       </c>
@@ -13711,7 +13768,7 @@
       </c>
       <c r="C32" s="2"/>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>30</v>
       </c>
@@ -13720,7 +13777,7 @@
       </c>
       <c r="C33" s="2"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <v>31</v>
       </c>
@@ -13728,7 +13785,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
         <v>32</v>
       </c>
@@ -13736,7 +13793,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>33</v>
       </c>
@@ -13744,7 +13801,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>34</v>
       </c>

</xml_diff>

<commit_message>
add lvl 40 sk ether npc
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/27_SiegeKitItem/SiegeKitItem.xlsx
+++ b/gu_in/Item.edf/27_SiegeKitItem/SiegeKitItem.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61877373-6E53-407C-946A-D19F0CEB61B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7B4B5FB-65C2-4EF3-850B-3D46CBFA5844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13477,6 +13477,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="40.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">

</xml_diff>

<commit_message>
ETHER NPC CHOOTY ADVANCED SK CHANGE TO 25% ATTACK
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/27_SiegeKitItem/SiegeKitItem.xlsx
+++ b/gu_in/Item.edf/27_SiegeKitItem/SiegeKitItem.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7B4B5FB-65C2-4EF3-850B-3D46CBFA5844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7A57A93-BFA6-4292-B8CC-0FD1900C2291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1632,7 +1632,7 @@
         <v>6</v>
       </c>
       <c r="AH4" s="3">
-        <v>0.34999999403953552</v>
+        <v>0.24999999403953599</v>
       </c>
       <c r="AI4" s="3">
         <v>0</v>
@@ -3162,7 +3162,7 @@
         <v>6</v>
       </c>
       <c r="AH14" s="3">
-        <v>0.34999999403953552</v>
+        <v>0.24999999403953599</v>
       </c>
       <c r="AI14" s="3">
         <v>0</v>
@@ -6977,7 +6977,7 @@
       </c>
       <c r="AT4">
         <f>SiegeKitItem!AH4</f>
-        <v>0.34999999403953552</v>
+        <v>0.24999999403953599</v>
       </c>
       <c r="AU4">
         <f>SiegeKitItem!AJ4</f>
@@ -9197,7 +9197,7 @@
       </c>
       <c r="AT14">
         <f>SiegeKitItem!AH14</f>
-        <v>0.34999999403953552</v>
+        <v>0.24999999403953599</v>
       </c>
       <c r="AU14">
         <f>SiegeKitItem!AJ14</f>

</xml_diff>